<commit_message>
feat: give the IEC examples the same ride-through curves as the WECC ones
</commit_message>
<xml_diff>
--- a/examples/Model/Wind/IECA2020WithProtections/Excel/Producer.xlsx
+++ b/examples/Model/Wind/IECA2020WithProtections/Excel/Producer.xlsx
@@ -8824,7 +8824,7 @@
         <v>628</v>
       </c>
       <c r="AF9" s="101">
-        <v>1.0</v>
+        <v>1.1</v>
       </c>
       <c r="AG9" s="98" t="s">
         <v>336</v>
@@ -8897,7 +8897,7 @@
         <v>635</v>
       </c>
       <c r="AF10" s="101">
-        <v>2.0</v>
+        <v>100.0</v>
       </c>
       <c r="AG10" s="98" t="s">
         <v>336</v>
@@ -8918,7 +8918,7 @@
         <v>637</v>
       </c>
       <c r="AF11" s="101">
-        <v>1.5</v>
+        <v>1.1001</v>
       </c>
       <c r="AG11" s="98" t="s">
         <v>336</v>
@@ -8939,7 +8939,7 @@
         <v>639</v>
       </c>
       <c r="AF12" s="101">
-        <v>2.0</v>
+        <v>30.0</v>
       </c>
       <c r="AG12" s="98" t="s">
         <v>336</v>
@@ -8960,7 +8960,7 @@
         <v>641</v>
       </c>
       <c r="AF13" s="101">
-        <v>2.0</v>
+        <v>1.15</v>
       </c>
       <c r="AG13" s="98" t="s">
         <v>336</v>
@@ -8981,7 +8981,7 @@
         <v>643</v>
       </c>
       <c r="AF14" s="101">
-        <v>2.0</v>
+        <v>30.0</v>
       </c>
       <c r="AG14" s="98" t="s">
         <v>336</v>
@@ -9001,7 +9001,9 @@
       <c r="AE15" s="98" t="s">
         <v>645</v>
       </c>
-      <c r="AF15" s="101"/>
+      <c r="AF15" s="101">
+        <v>1.1501</v>
+      </c>
       <c r="AG15" s="98" t="s">
         <v>336</v>
       </c>
@@ -9020,7 +9022,9 @@
       <c r="AE16" s="98" t="s">
         <v>647</v>
       </c>
-      <c r="AF16" s="101"/>
+      <c r="AF16" s="101">
+        <v>2.5</v>
+      </c>
       <c r="AG16" s="98" t="s">
         <v>336</v>
       </c>
@@ -9039,7 +9043,9 @@
       <c r="AE17" s="98" t="s">
         <v>649</v>
       </c>
-      <c r="AF17" s="101"/>
+      <c r="AF17" s="101">
+        <v>1.25</v>
+      </c>
       <c r="AG17" s="98" t="s">
         <v>336</v>
       </c>
@@ -9058,7 +9064,9 @@
       <c r="AE18" s="98" t="s">
         <v>651</v>
       </c>
-      <c r="AF18" s="101"/>
+      <c r="AF18" s="101">
+        <v>2.5</v>
+      </c>
       <c r="AG18" s="98" t="s">
         <v>336</v>
       </c>
@@ -9077,7 +9085,9 @@
       <c r="AE19" s="98" t="s">
         <v>653</v>
       </c>
-      <c r="AF19" s="101"/>
+      <c r="AF19" s="101">
+        <v>1.2501</v>
+      </c>
       <c r="AG19" s="98" t="s">
         <v>336</v>
       </c>
@@ -9096,7 +9106,9 @@
       <c r="AE20" s="98" t="s">
         <v>655</v>
       </c>
-      <c r="AF20" s="101"/>
+      <c r="AF20" s="101">
+        <v>0.1</v>
+      </c>
       <c r="AG20" s="98" t="s">
         <v>336</v>
       </c>
@@ -9115,7 +9127,9 @@
       <c r="AE21" s="98" t="s">
         <v>657</v>
       </c>
-      <c r="AF21" s="101"/>
+      <c r="AF21" s="101">
+        <v>1.3</v>
+      </c>
       <c r="AG21" s="98" t="s">
         <v>336</v>
       </c>
@@ -9134,7 +9148,9 @@
       <c r="AE22" s="98" t="s">
         <v>659</v>
       </c>
-      <c r="AF22" s="101"/>
+      <c r="AF22" s="101">
+        <v>0.1</v>
+      </c>
       <c r="AG22" s="98" t="s">
         <v>336</v>
       </c>
@@ -9215,7 +9231,7 @@
         <v>667</v>
       </c>
       <c r="AF26" s="101">
-        <v>2.0</v>
+        <v>1.5</v>
       </c>
       <c r="AG26" s="98" t="s">
         <v>336</v>
@@ -9236,7 +9252,7 @@
         <v>669</v>
       </c>
       <c r="AF27" s="101">
-        <v>0.5</v>
+        <v>0.8499</v>
       </c>
       <c r="AG27" s="98" t="s">
         <v>336</v>
@@ -9257,7 +9273,7 @@
         <v>671</v>
       </c>
       <c r="AF28" s="101">
-        <v>2.0</v>
+        <v>1.5</v>
       </c>
       <c r="AG28" s="98" t="s">
         <v>336</v>
@@ -9278,7 +9294,7 @@
         <v>673</v>
       </c>
       <c r="AF29" s="101">
-        <v>1.0</v>
+        <v>0.85</v>
       </c>
       <c r="AG29" s="98" t="s">
         <v>336</v>
@@ -9299,7 +9315,7 @@
         <v>675</v>
       </c>
       <c r="AF30" s="101">
-        <v>2.0</v>
+        <v>30.0</v>
       </c>
       <c r="AG30" s="98" t="s">
         <v>336</v>
@@ -9319,7 +9335,9 @@
       <c r="AE31" s="98" t="s">
         <v>677</v>
       </c>
-      <c r="AF31" s="101"/>
+      <c r="AF31" s="101">
+        <v>0.8999</v>
+      </c>
       <c r="AG31" s="98" t="s">
         <v>336</v>
       </c>
@@ -9338,7 +9356,9 @@
       <c r="AE32" s="98" t="s">
         <v>679</v>
       </c>
-      <c r="AF32" s="101"/>
+      <c r="AF32" s="101">
+        <v>30.0</v>
+      </c>
       <c r="AG32" s="98" t="s">
         <v>336</v>
       </c>
@@ -9357,7 +9377,9 @@
       <c r="AE33" s="98" t="s">
         <v>681</v>
       </c>
-      <c r="AF33" s="101"/>
+      <c r="AF33" s="101">
+        <v>0.9</v>
+      </c>
       <c r="AG33" s="98" t="s">
         <v>336</v>
       </c>
@@ -9376,7 +9398,9 @@
       <c r="AE34" s="98" t="s">
         <v>683</v>
       </c>
-      <c r="AF34" s="101"/>
+      <c r="AF34" s="101">
+        <v>100.0</v>
+      </c>
       <c r="AG34" s="98" t="s">
         <v>336</v>
       </c>

</xml_diff>

<commit_message>
feat: write the ride-through overvoltage curve as a ramp instead of a staircase
</commit_message>
<xml_diff>
--- a/examples/Model/Wind/IECA2020WithProtections/Excel/Producer.xlsx
+++ b/examples/Model/Wind/IECA2020WithProtections/Excel/Producer.xlsx
@@ -8939,7 +8939,7 @@
         <v>639</v>
       </c>
       <c r="AF12" s="101">
-        <v>30.0</v>
+        <v>30.1</v>
       </c>
       <c r="AG12" s="98" t="s">
         <v>336</v>
@@ -8960,7 +8960,7 @@
         <v>641</v>
       </c>
       <c r="AF13" s="101">
-        <v>1.15</v>
+        <v>1.1999</v>
       </c>
       <c r="AG13" s="98" t="s">
         <v>336</v>
@@ -8981,7 +8981,7 @@
         <v>643</v>
       </c>
       <c r="AF14" s="101">
-        <v>30.0</v>
+        <v>30.1</v>
       </c>
       <c r="AG14" s="98" t="s">
         <v>336</v>
@@ -9002,7 +9002,7 @@
         <v>645</v>
       </c>
       <c r="AF15" s="101">
-        <v>1.1501</v>
+        <v>1.2001</v>
       </c>
       <c r="AG15" s="98" t="s">
         <v>336</v>
@@ -9023,7 +9023,7 @@
         <v>647</v>
       </c>
       <c r="AF16" s="101">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="AG16" s="98" t="s">
         <v>336</v>
@@ -9044,7 +9044,7 @@
         <v>649</v>
       </c>
       <c r="AF17" s="101">
-        <v>1.25</v>
+        <v>1.2749</v>
       </c>
       <c r="AG17" s="98" t="s">
         <v>336</v>
@@ -9065,7 +9065,7 @@
         <v>651</v>
       </c>
       <c r="AF18" s="101">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="AG18" s="98" t="s">
         <v>336</v>
@@ -9086,7 +9086,7 @@
         <v>653</v>
       </c>
       <c r="AF19" s="101">
-        <v>1.2501</v>
+        <v>1.2751</v>
       </c>
       <c r="AG19" s="98" t="s">
         <v>336</v>
@@ -9107,7 +9107,7 @@
         <v>655</v>
       </c>
       <c r="AF20" s="101">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="AG20" s="98" t="s">
         <v>336</v>
@@ -9149,7 +9149,7 @@
         <v>659</v>
       </c>
       <c r="AF22" s="101">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="AG22" s="98" t="s">
         <v>336</v>

</xml_diff>

<commit_message>
feat: set the ride-through curves to RTE's times, written as continuous curves
</commit_message>
<xml_diff>
--- a/examples/Model/Wind/IECA2020WithProtections/Excel/Producer.xlsx
+++ b/examples/Model/Wind/IECA2020WithProtections/Excel/Producer.xlsx
@@ -8897,7 +8897,7 @@
         <v>635</v>
       </c>
       <c r="AF10" s="101">
-        <v>100.0</v>
+        <v>100.005</v>
       </c>
       <c r="AG10" s="98" t="s">
         <v>336</v>
@@ -8918,7 +8918,7 @@
         <v>637</v>
       </c>
       <c r="AF11" s="101">
-        <v>1.1001</v>
+        <v>1.15</v>
       </c>
       <c r="AG11" s="98" t="s">
         <v>336</v>
@@ -8939,7 +8939,7 @@
         <v>639</v>
       </c>
       <c r="AF12" s="101">
-        <v>30.1</v>
+        <v>30.005</v>
       </c>
       <c r="AG12" s="98" t="s">
         <v>336</v>
@@ -8960,7 +8960,7 @@
         <v>641</v>
       </c>
       <c r="AF13" s="101">
-        <v>1.1999</v>
+        <v>1.25</v>
       </c>
       <c r="AG13" s="98" t="s">
         <v>336</v>
@@ -8981,7 +8981,7 @@
         <v>643</v>
       </c>
       <c r="AF14" s="101">
-        <v>30.1</v>
+        <v>2.505</v>
       </c>
       <c r="AG14" s="98" t="s">
         <v>336</v>
@@ -9002,7 +9002,7 @@
         <v>645</v>
       </c>
       <c r="AF15" s="101">
-        <v>1.2001</v>
+        <v>1.3</v>
       </c>
       <c r="AG15" s="98" t="s">
         <v>336</v>
@@ -9023,7 +9023,7 @@
         <v>647</v>
       </c>
       <c r="AF16" s="101">
-        <v>2.6</v>
+        <v>0.105</v>
       </c>
       <c r="AG16" s="98" t="s">
         <v>336</v>
@@ -9044,7 +9044,7 @@
         <v>649</v>
       </c>
       <c r="AF17" s="101">
-        <v>1.2749</v>
+        <v>1.4</v>
       </c>
       <c r="AG17" s="98" t="s">
         <v>336</v>
@@ -9065,7 +9065,7 @@
         <v>651</v>
       </c>
       <c r="AF18" s="101">
-        <v>2.6</v>
+        <v>0.105</v>
       </c>
       <c r="AG18" s="98" t="s">
         <v>336</v>
@@ -9231,7 +9231,7 @@
         <v>667</v>
       </c>
       <c r="AF26" s="101">
-        <v>1.5</v>
+        <v>0.1505</v>
       </c>
       <c r="AG26" s="98" t="s">
         <v>336</v>
@@ -9252,7 +9252,7 @@
         <v>669</v>
       </c>
       <c r="AF27" s="101">
-        <v>0.8499</v>
+        <v>0.85</v>
       </c>
       <c r="AG27" s="98" t="s">
         <v>336</v>
@@ -9273,7 +9273,7 @@
         <v>671</v>
       </c>
       <c r="AF28" s="101">
-        <v>1.5</v>
+        <v>30.005</v>
       </c>
       <c r="AG28" s="98" t="s">
         <v>336</v>
@@ -9294,7 +9294,7 @@
         <v>673</v>
       </c>
       <c r="AF29" s="101">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="AG29" s="98" t="s">
         <v>336</v>
@@ -9315,7 +9315,7 @@
         <v>675</v>
       </c>
       <c r="AF30" s="101">
-        <v>30.0</v>
+        <v>100.005</v>
       </c>
       <c r="AG30" s="98" t="s">
         <v>336</v>

</xml_diff>

<commit_message>
feat: set the ride-through curves to the times RTE's grid code gives, with its margin
</commit_message>
<xml_diff>
--- a/examples/Model/Wind/IECA2020WithProtections/Excel/Producer.xlsx
+++ b/examples/Model/Wind/IECA2020WithProtections/Excel/Producer.xlsx
@@ -8905,7 +8905,7 @@
         <v>640</v>
       </c>
       <c r="AF10" s="101">
-        <v>100.005</v>
+        <v>100.0</v>
       </c>
       <c r="AG10" s="98" t="s">
         <v>330</v>
@@ -8947,7 +8947,7 @@
         <v>644</v>
       </c>
       <c r="AF12" s="101">
-        <v>30.005</v>
+        <v>30.1</v>
       </c>
       <c r="AG12" s="98" t="s">
         <v>330</v>
@@ -8989,7 +8989,7 @@
         <v>648</v>
       </c>
       <c r="AF14" s="101">
-        <v>2.505</v>
+        <v>2.6</v>
       </c>
       <c r="AG14" s="98" t="s">
         <v>330</v>
@@ -9031,7 +9031,7 @@
         <v>652</v>
       </c>
       <c r="AF16" s="101">
-        <v>0.105</v>
+        <v>0.2</v>
       </c>
       <c r="AG16" s="98" t="s">
         <v>330</v>
@@ -9073,7 +9073,7 @@
         <v>656</v>
       </c>
       <c r="AF18" s="101">
-        <v>0.105</v>
+        <v>0.2</v>
       </c>
       <c r="AG18" s="98" t="s">
         <v>330</v>
@@ -9239,7 +9239,7 @@
         <v>672</v>
       </c>
       <c r="AF26" s="101">
-        <v>0.1505</v>
+        <v>0.25</v>
       </c>
       <c r="AG26" s="98" t="s">
         <v>330</v>
@@ -9281,7 +9281,7 @@
         <v>676</v>
       </c>
       <c r="AF28" s="101">
-        <v>30.005</v>
+        <v>30.1</v>
       </c>
       <c r="AG28" s="98" t="s">
         <v>330</v>
@@ -9323,7 +9323,7 @@
         <v>680</v>
       </c>
       <c r="AF30" s="101">
-        <v>100.005</v>
+        <v>100.0</v>
       </c>
       <c r="AG30" s="98" t="s">
         <v>330</v>

</xml_diff>

<commit_message>
fix: keep the IEC ride-through tables strictly increasing
</commit_message>
<xml_diff>
--- a/examples/Model/Wind/IECA2020WithProtections/Excel/Producer.xlsx
+++ b/examples/Model/Wind/IECA2020WithProtections/Excel/Producer.xlsx
@@ -9093,9 +9093,7 @@
       <c r="AE19" s="98" t="s">
         <v>658</v>
       </c>
-      <c r="AF19" s="101">
-        <v>1.2751</v>
-      </c>
+      <c r="AF19" s="101"/>
       <c r="AG19" s="98" t="s">
         <v>330</v>
       </c>
@@ -9114,9 +9112,7 @@
       <c r="AE20" s="98" t="s">
         <v>660</v>
       </c>
-      <c r="AF20" s="101">
-        <v>0.15</v>
-      </c>
+      <c r="AF20" s="101"/>
       <c r="AG20" s="98" t="s">
         <v>330</v>
       </c>
@@ -9135,9 +9131,7 @@
       <c r="AE21" s="98" t="s">
         <v>662</v>
       </c>
-      <c r="AF21" s="101">
-        <v>1.3</v>
-      </c>
+      <c r="AF21" s="101"/>
       <c r="AG21" s="98" t="s">
         <v>330</v>
       </c>
@@ -9156,9 +9150,7 @@
       <c r="AE22" s="98" t="s">
         <v>664</v>
       </c>
-      <c r="AF22" s="101">
-        <v>0.15</v>
-      </c>
+      <c r="AF22" s="101"/>
       <c r="AG22" s="98" t="s">
         <v>330</v>
       </c>
@@ -9343,9 +9335,7 @@
       <c r="AE31" s="98" t="s">
         <v>682</v>
       </c>
-      <c r="AF31" s="101">
-        <v>0.8999</v>
-      </c>
+      <c r="AF31" s="101"/>
       <c r="AG31" s="98" t="s">
         <v>330</v>
       </c>
@@ -9364,9 +9354,7 @@
       <c r="AE32" s="98" t="s">
         <v>684</v>
       </c>
-      <c r="AF32" s="101">
-        <v>30.0</v>
-      </c>
+      <c r="AF32" s="101"/>
       <c r="AG32" s="98" t="s">
         <v>330</v>
       </c>
@@ -9385,9 +9373,7 @@
       <c r="AE33" s="98" t="s">
         <v>686</v>
       </c>
-      <c r="AF33" s="101">
-        <v>0.9</v>
-      </c>
+      <c r="AF33" s="101"/>
       <c r="AG33" s="98" t="s">
         <v>330</v>
       </c>
@@ -9406,9 +9392,7 @@
       <c r="AE34" s="98" t="s">
         <v>688</v>
       </c>
-      <c r="AF34" s="101">
-        <v>100.0</v>
-      </c>
+      <c r="AF34" s="101"/>
       <c r="AG34" s="98" t="s">
         <v>330</v>
       </c>

</xml_diff>

<commit_message>
feat: carry RTE's ride-through tables as the grid code writes them
</commit_message>
<xml_diff>
--- a/examples/Model/Wind/IECA2020WithProtections/Excel/Producer.xlsx
+++ b/examples/Model/Wind/IECA2020WithProtections/Excel/Producer.xlsx
@@ -8926,7 +8926,7 @@
         <v>642</v>
       </c>
       <c r="AF11" s="101">
-        <v>1.15</v>
+        <v>1.1001</v>
       </c>
       <c r="AG11" s="98" t="s">
         <v>330</v>
@@ -8968,7 +8968,7 @@
         <v>646</v>
       </c>
       <c r="AF13" s="101">
-        <v>1.25</v>
+        <v>1.15</v>
       </c>
       <c r="AG13" s="98" t="s">
         <v>330</v>
@@ -8989,7 +8989,7 @@
         <v>648</v>
       </c>
       <c r="AF14" s="101">
-        <v>2.6</v>
+        <v>30.1</v>
       </c>
       <c r="AG14" s="98" t="s">
         <v>330</v>
@@ -9010,7 +9010,7 @@
         <v>650</v>
       </c>
       <c r="AF15" s="101">
-        <v>1.3</v>
+        <v>1.1501</v>
       </c>
       <c r="AG15" s="98" t="s">
         <v>330</v>
@@ -9031,7 +9031,7 @@
         <v>652</v>
       </c>
       <c r="AF16" s="101">
-        <v>0.2</v>
+        <v>2.6</v>
       </c>
       <c r="AG16" s="98" t="s">
         <v>330</v>
@@ -9052,7 +9052,7 @@
         <v>654</v>
       </c>
       <c r="AF17" s="101">
-        <v>1.4</v>
+        <v>1.25</v>
       </c>
       <c r="AG17" s="98" t="s">
         <v>330</v>
@@ -9073,7 +9073,7 @@
         <v>656</v>
       </c>
       <c r="AF18" s="101">
-        <v>0.2</v>
+        <v>2.6</v>
       </c>
       <c r="AG18" s="98" t="s">
         <v>330</v>
@@ -9093,7 +9093,9 @@
       <c r="AE19" s="98" t="s">
         <v>658</v>
       </c>
-      <c r="AF19" s="101"/>
+      <c r="AF19" s="101">
+        <v>1.2501</v>
+      </c>
       <c r="AG19" s="98" t="s">
         <v>330</v>
       </c>
@@ -9112,7 +9114,9 @@
       <c r="AE20" s="98" t="s">
         <v>660</v>
       </c>
-      <c r="AF20" s="101"/>
+      <c r="AF20" s="101">
+        <v>0.2</v>
+      </c>
       <c r="AG20" s="98" t="s">
         <v>330</v>
       </c>
@@ -9131,7 +9135,9 @@
       <c r="AE21" s="98" t="s">
         <v>662</v>
       </c>
-      <c r="AF21" s="101"/>
+      <c r="AF21" s="101">
+        <v>1.3</v>
+      </c>
       <c r="AG21" s="98" t="s">
         <v>330</v>
       </c>
@@ -9150,7 +9156,9 @@
       <c r="AE22" s="98" t="s">
         <v>664</v>
       </c>
-      <c r="AF22" s="101"/>
+      <c r="AF22" s="101">
+        <v>0.2</v>
+      </c>
       <c r="AG22" s="98" t="s">
         <v>330</v>
       </c>
@@ -9252,7 +9260,7 @@
         <v>674</v>
       </c>
       <c r="AF27" s="101">
-        <v>0.85</v>
+        <v>0.8499</v>
       </c>
       <c r="AG27" s="98" t="s">
         <v>330</v>
@@ -9273,7 +9281,7 @@
         <v>676</v>
       </c>
       <c r="AF28" s="101">
-        <v>30.1</v>
+        <v>1.6</v>
       </c>
       <c r="AG28" s="98" t="s">
         <v>330</v>
@@ -9294,7 +9302,7 @@
         <v>678</v>
       </c>
       <c r="AF29" s="101">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="AG29" s="98" t="s">
         <v>330</v>
@@ -9315,7 +9323,7 @@
         <v>680</v>
       </c>
       <c r="AF30" s="101">
-        <v>100.0</v>
+        <v>30.1</v>
       </c>
       <c r="AG30" s="98" t="s">
         <v>330</v>
@@ -9335,7 +9343,9 @@
       <c r="AE31" s="98" t="s">
         <v>682</v>
       </c>
-      <c r="AF31" s="101"/>
+      <c r="AF31" s="101">
+        <v>0.8999</v>
+      </c>
       <c r="AG31" s="98" t="s">
         <v>330</v>
       </c>
@@ -9354,7 +9364,9 @@
       <c r="AE32" s="98" t="s">
         <v>684</v>
       </c>
-      <c r="AF32" s="101"/>
+      <c r="AF32" s="101">
+        <v>30.1</v>
+      </c>
       <c r="AG32" s="98" t="s">
         <v>330</v>
       </c>
@@ -9373,7 +9385,9 @@
       <c r="AE33" s="98" t="s">
         <v>686</v>
       </c>
-      <c r="AF33" s="101"/>
+      <c r="AF33" s="101">
+        <v>0.9</v>
+      </c>
       <c r="AG33" s="98" t="s">
         <v>330</v>
       </c>
@@ -9392,7 +9406,9 @@
       <c r="AE34" s="98" t="s">
         <v>688</v>
       </c>
-      <c r="AF34" s="101"/>
+      <c r="AF34" s="101">
+        <v>100.0</v>
+      </c>
       <c r="AG34" s="98" t="s">
         <v>330</v>
       </c>

</xml_diff>